<commit_message>
scan: seg8 2026-08-06 18:47 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq0_2026-08-06.xlsx
+++ b/output/full_scan/batch_seq0_2026-08-06.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O116"/>
+  <dimension ref="A1:O117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5096,7 +5096,7 @@
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>211.8555816657334</v>
+        <v>211.8555816657333</v>
       </c>
       <c r="E88" s="2" t="n">
         <v>15.7</v>
@@ -5721,21 +5721,21 @@
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>8463</v>
+        <v>8291</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>潤泰材</t>
+          <t>尚茂</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>161.4710593157427</v>
+        <v>162.3482270222162</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>20.9</v>
+        <v>41</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,13 +5746,13 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>39.96203152495536</v>
+        <v>51.64232728927961</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>22.22818396417805</v>
+        <v>17.31844030746549</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>1.266036570935546</v>
+        <v>1.264771638454168</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.0315341259819035</v>
+        <v>0.864239518879423</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>8201</v>
+        <v>8463</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>無敵</t>
+          <t>潤泰材</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>153.0833145496608</v>
+        <v>161.4710593157427</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>11.85</v>
+        <v>20.9</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,13 +5799,13 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>41.45194258422832</v>
+        <v>39.96203152495536</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>27.29063901284414</v>
+        <v>22.22818396417805</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0.5003096098915366</v>
+        <v>1.266036570935546</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>0</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.009539153292022399</v>
+        <v>-0.0315341259819035</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5827,21 +5827,21 @@
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>8072</v>
+        <v>8201</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>陞泰</t>
+          <t>無敵</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>152.4279261332632</v>
+        <v>153.0833145496608</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>26.2</v>
+        <v>11.85</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,13 +5852,13 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>40.02614586602942</v>
+        <v>41.45194258422832</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>18.85194141603574</v>
+        <v>27.29063901284414</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>1.201002637853382</v>
+        <v>0.5003096098915366</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>0</v>
@@ -5870,31 +5870,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>0.0031209569624772</v>
+        <v>-0.009539153292022399</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>9902</v>
+        <v>8072</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>台火</t>
+          <t>陞泰</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>151.5889144445392</v>
+        <v>152.4279261332632</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>13.65</v>
+        <v>26.2</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,13 +5905,13 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>48.28544206499284</v>
+        <v>40.02614586602942</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>8.380322107333814</v>
+        <v>18.85194141603574</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>1.004579451418339</v>
+        <v>1.201002637853382</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>0</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>0.0041992039765893</v>
+        <v>0.0031209569624772</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5933,21 +5933,21 @@
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>8054</v>
+        <v>9902</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>安國</t>
+          <t>台火</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>149.8287594736743</v>
+        <v>151.5889144445392</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>83.40000000000001</v>
+        <v>13.65</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,13 +5958,13 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>39.49690961427798</v>
+        <v>48.28544206499284</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>24.08835611601837</v>
+        <v>8.380322107333814</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>0.5496299693112824</v>
+        <v>1.004579451418339</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.2505530324846479</v>
+        <v>0.0041992039765893</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>8341</v>
+        <v>8054</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>日友</t>
+          <t>安國</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>147.7904802489459</v>
+        <v>149.8287594736743</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>75.3</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,13 +6011,13 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>42.56493327103789</v>
+        <v>39.49690961427798</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>13.46329652768679</v>
+        <v>24.08835611601837</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>0.3995782710820679</v>
+        <v>0.5496299693112824</v>
       </c>
       <c r="K105" s="2" t="n">
         <v>0</v>
@@ -6029,31 +6029,31 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.0762285555039223</v>
+        <v>-0.2505530324846479</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>8097</v>
+        <v>8341</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>常珵</t>
+          <t>日友</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>146.3648609597032</v>
+        <v>147.7904802489459</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>51.8</v>
+        <v>75.3</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,13 +6064,13 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>39.46196542572187</v>
+        <v>42.56493327103789</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>14.02442123297152</v>
+        <v>13.46329652768679</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>0.4156112194532448</v>
+        <v>0.3995782710820679</v>
       </c>
       <c r="K106" s="2" t="n">
         <v>0</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.1373995393204576</v>
+        <v>-0.0762285555039223</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6092,21 +6092,21 @@
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>8940</v>
+        <v>8097</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>新天地</t>
+          <t>常珵</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>139.7538275331472</v>
+        <v>146.3648609597032</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>15.35</v>
+        <v>51.8</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,13 +6117,13 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>26.0091718586589</v>
+        <v>39.46196542572187</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>16.71545150302683</v>
+        <v>14.02442123297152</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>0.4870141824879453</v>
+        <v>0.4156112194532448</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.0535666182412102</v>
+        <v>0.1373995393204576</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6145,21 +6145,21 @@
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>8472</v>
+        <v>8940</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>夠麻吉</t>
+          <t>新天地</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>127.8620783467132</v>
+        <v>139.7538275331472</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>68</v>
+        <v>15.35</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,13 +6170,13 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>34.31294828444095</v>
+        <v>26.0091718586589</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>17.19842493629408</v>
+        <v>16.71545150302683</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>0.199008741527579</v>
+        <v>0.4870141824879453</v>
       </c>
       <c r="K108" s="2" t="n">
         <v>0</v>
@@ -6188,31 +6188,31 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.1616349399993684</v>
+        <v>-0.0535666182412102</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>8092</v>
+        <v>8472</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>建暐</t>
+          <t>夠麻吉</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>105.457422433168</v>
+        <v>127.8620783467132</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>13.4</v>
+        <v>68</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,13 +6223,13 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>44.23751853290251</v>
+        <v>34.31294828444095</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>14.96683007437636</v>
+        <v>17.19842493629408</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>0.3756800547171661</v>
+        <v>0.199008741527579</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>0</v>
@@ -6241,31 +6241,31 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.0543748358057344</v>
+        <v>-0.1616349399993684</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>8104</v>
+        <v>8092</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>錸寶</t>
+          <t>建暐</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>101.6916263052699</v>
+        <v>105.457422433168</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>31.15</v>
+        <v>13.4</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,13 +6276,13 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>38.65516150666387</v>
+        <v>44.23751853290251</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>31.29975883825493</v>
+        <v>14.96683007437636</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>0.3373780161006777</v>
+        <v>0.3756800547171661</v>
       </c>
       <c r="K110" s="2" t="n">
         <v>0</v>
@@ -6294,31 +6294,31 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.1040917479170095</v>
+        <v>0.0543748358057344</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>8277</v>
+        <v>8104</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>商丞</t>
+          <t>錸寶</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>87.16903742846229</v>
+        <v>101.6916263052699</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>8.119999999999999</v>
+        <v>31.15</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,13 +6329,13 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>44.30594360208702</v>
+        <v>38.65516150666387</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>18.42631541925521</v>
+        <v>31.29975883825493</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.2483562115201599</v>
+        <v>0.3373780161006777</v>
       </c>
       <c r="K111" s="2" t="n">
         <v>0</v>
@@ -6347,31 +6347,31 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.058976168254979</v>
+        <v>-0.1040917479170095</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, mfi_strong</t>
+          <t>market_above_ma60, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>8431</v>
+        <v>8277</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>匯鑽科</t>
+          <t>商丞</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>85.7558926529817</v>
+        <v>87.16903742846229</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>50</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,13 +6382,13 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>51.69962131927152</v>
+        <v>44.30594360208702</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>17.81268676983301</v>
+        <v>18.42631541925521</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.3839974717522516</v>
+        <v>0.2483562115201599</v>
       </c>
       <c r="K112" s="2" t="n">
         <v>0</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.6305387439754309</v>
+        <v>0.058976168254979</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6410,21 +6410,21 @@
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>8085</v>
+        <v>8431</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>福華</t>
+          <t>匯鑽科</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>81.35755624733011</v>
+        <v>85.7558926529817</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>11.15</v>
+        <v>50</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,16 +6435,16 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>43.53335199749232</v>
+        <v>51.69962131927152</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>14.81749261882666</v>
+        <v>17.81268676983301</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.6897068950419826</v>
+        <v>0.3839974717522516</v>
       </c>
       <c r="K113" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L113" s="2" t="n">
         <v>0</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.0116250476994556</v>
+        <v>0.6305387439754309</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>8176</v>
+        <v>8085</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>智捷</t>
+          <t>福華</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>66.58767673422321</v>
+        <v>81.35755624733011</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>9.83</v>
+        <v>11.15</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,16 +6488,16 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>43.76062387188076</v>
+        <v>43.53335199749232</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>10.39320101292088</v>
+        <v>14.81749261882666</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.1799290400202327</v>
+        <v>0.6897068950419826</v>
       </c>
       <c r="K114" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L114" s="2" t="n">
         <v>0</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.0039152099670361</v>
+        <v>0.0116250476994556</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6516,21 +6516,21 @@
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>9906</v>
+        <v>8176</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>欣巴巴</t>
+          <t>智捷</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>61.70488338832586</v>
+        <v>66.58767673422321</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>39</v>
+        <v>9.83</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,13 +6541,13 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>44.00728483259322</v>
+        <v>43.76062387188076</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>11.51247174346926</v>
+        <v>10.39320101292088</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>0.5054175002599628</v>
+        <v>0.1799290400202327</v>
       </c>
       <c r="K115" s="2" t="n">
         <v>0</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.1084879186712785</v>
+        <v>-0.0039152099670361</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6569,52 +6569,105 @@
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
+        <v>9906</v>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>欣巴巴</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D116" s="2" t="n">
+        <v>61.70488338832586</v>
+      </c>
+      <c r="E116" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H116" s="2" t="n">
+        <v>44.00728483259322</v>
+      </c>
+      <c r="I116" s="2" t="n">
+        <v>11.51247174346926</v>
+      </c>
+      <c r="J116" s="2" t="n">
+        <v>0.5054175002599628</v>
+      </c>
+      <c r="K116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M116" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N116" s="2" t="n">
+        <v>-0.1084879186712785</v>
+      </c>
+      <c r="O116" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="n">
         <v>8084</v>
       </c>
-      <c r="B116" s="2" t="inlineStr">
+      <c r="B117" s="2" t="inlineStr">
         <is>
           <t>巨虹</t>
         </is>
       </c>
-      <c r="C116" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D116" s="2" t="n">
+      <c r="C117" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D117" s="2" t="n">
         <v>50.4810482790589</v>
       </c>
-      <c r="E116" s="2" t="n">
+      <c r="E117" s="2" t="n">
         <v>42.45</v>
       </c>
-      <c r="F116" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="G116" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H116" s="2" t="n">
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="G117" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H117" s="2" t="n">
         <v>41.90347970197072</v>
       </c>
-      <c r="I116" s="2" t="n">
+      <c r="I117" s="2" t="n">
         <v>17.67365369366864</v>
       </c>
-      <c r="J116" s="2" t="n">
+      <c r="J117" s="2" t="n">
         <v>0.3211234059409245</v>
       </c>
-      <c r="K116" s="2" t="n">
+      <c r="K117" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L116" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M116" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N116" s="2" t="n">
+      <c r="L117" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M117" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N117" s="2" t="n">
         <v>-0.08971935772277261</v>
       </c>
-      <c r="O116" s="2" t="inlineStr">
+      <c r="O117" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase</t>
         </is>

</xml_diff>